<commit_message>
Figure updates (05/22/25 draft)
</commit_message>
<xml_diff>
--- a/RT_qPCR/qPCR_PossibleDC_EVEs.xlsx
+++ b/RT_qPCR/qPCR_PossibleDC_EVEs.xlsx
@@ -1,21 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10309"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lexikeene/Documents/Research/diverse_collections/github/RT_qPCR/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA793FD5-5269-E741-92EC-038199A411B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41B39F64-A310-5046-9305-4326E822A74E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1560" yWindow="760" windowWidth="28680" windowHeight="17160" activeTab="1" xr2:uid="{B8C42D12-2C26-4FF1-BD45-0920706209D2}"/>
+    <workbookView xWindow="30400" yWindow="500" windowWidth="38080" windowHeight="19400" activeTab="3" xr2:uid="{B8C42D12-2C26-4FF1-BD45-0920706209D2}"/>
   </bookViews>
   <sheets>
     <sheet name="qPCR" sheetId="4" r:id="rId1"/>
     <sheet name="EVE Specific PCR" sheetId="6" r:id="rId2"/>
     <sheet name="Platemaps" sheetId="5" r:id="rId3"/>
+    <sheet name="Sanger_Seq" sheetId="7" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1461" uniqueCount="612">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1538" uniqueCount="645">
   <si>
     <t>1x</t>
   </si>
@@ -1914,12 +1915,111 @@
       <t>: I am using this protocol to screen the potential EVE positive samples using Ali's EVE genotyping primers. I will be running this PCR on 03/14/2025 and the gel on 03/15/2025.</t>
     </r>
   </si>
+  <si>
+    <t>Sample Name</t>
+  </si>
+  <si>
+    <t>qPCR Plate Location</t>
+  </si>
+  <si>
+    <t>500-F-8</t>
+  </si>
+  <si>
+    <t>500-F-27</t>
+  </si>
+  <si>
+    <t>500-F-67</t>
+  </si>
+  <si>
+    <t>1020-0818-E4</t>
+  </si>
+  <si>
+    <t>1020-C1</t>
+  </si>
+  <si>
+    <t>1020-E5</t>
+  </si>
+  <si>
+    <t>1020-F5</t>
+  </si>
+  <si>
+    <t>1020-F6</t>
+  </si>
+  <si>
+    <t>1020-M-15</t>
+  </si>
+  <si>
+    <t>1020-M-16</t>
+  </si>
+  <si>
+    <t>1428-M-1</t>
+  </si>
+  <si>
+    <t>1428-M-42</t>
+  </si>
+  <si>
+    <t>Myrtle-E4</t>
+  </si>
+  <si>
+    <t>Myrtle-E5</t>
+  </si>
+  <si>
+    <t>Gel Result</t>
+  </si>
+  <si>
+    <t>high</t>
+  </si>
+  <si>
+    <t>medium</t>
+  </si>
+  <si>
+    <t>low</t>
+  </si>
+  <si>
+    <t>Sequencing Result</t>
+  </si>
+  <si>
+    <t>Drosophila melanogaster X BAC RP98-12H1</t>
+  </si>
+  <si>
+    <t>Accession</t>
+  </si>
+  <si>
+    <t>AC023691.3</t>
+  </si>
+  <si>
+    <t>OR729115.1</t>
+  </si>
+  <si>
+    <t>MAG: Galbut virus isolate MD_FoCo21_19 segment RNA1, complete sequence</t>
+  </si>
+  <si>
+    <t>Drosophila melanogaster 3L BAC RP98-26L14</t>
+  </si>
+  <si>
+    <t>AC010058.7</t>
+  </si>
+  <si>
+    <t>Galbut virus isolate 1004283 putative RNA-dependent RNA polymerase gene, complete cds</t>
+  </si>
+  <si>
+    <t>OR820569.1</t>
+  </si>
+  <si>
+    <t>% Identity</t>
+  </si>
+  <si>
+    <t>FAILED</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="20" x14ac:knownFonts="1">
+  <fonts count="22" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2053,6 +2153,21 @@
     </font>
     <font>
       <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -2215,10 +2330,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="62">
+  <cellXfs count="67">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -2337,29 +2453,25 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="14" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2370,11 +2482,29 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -2447,6 +2577,1040 @@
         </a:prstGeom>
       </xdr:spPr>
     </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>213398</xdr:colOff>
+      <xdr:row>38</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{382C1C42-351F-67AE-546B-0704A8CED02C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5471583" y="0"/>
+          <a:ext cx="8468398" cy="7260167"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>237067</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>177800</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>575734</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>61383</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="4" name="TextBox 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0159BD36-5AAD-8391-79F6-E4DAE68A8142}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6574367" y="1511300"/>
+          <a:ext cx="338667" cy="264583"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525" cmpd="sng">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="bg1">
+                  <a:lumMod val="95000"/>
+                </a:schemeClr>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>A3</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>749301</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>2116</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>262468</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>76199</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="5" name="TextBox 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CECFD09C-C808-F24B-804C-6AC3507751DF}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="7086601" y="1526116"/>
+          <a:ext cx="338667" cy="264583"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525" cmpd="sng">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="bg1">
+                  <a:lumMod val="95000"/>
+                </a:schemeClr>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>A5</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>645584</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>150282</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>234950</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>33865</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="6" name="TextBox 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{37A13C11-D2AB-B048-891D-71B0671AE5A1}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="8633884" y="1483782"/>
+          <a:ext cx="414866" cy="264583"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525" cmpd="sng">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="bg1">
+                  <a:lumMod val="95000"/>
+                </a:schemeClr>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>A11</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>419101</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>148166</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>755651</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>31749</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="7" name="TextBox 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A04E7331-8D3B-144D-8FA3-A693B3C3A1F7}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9232901" y="1481666"/>
+          <a:ext cx="336550" cy="264583"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525" cmpd="sng">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="bg1">
+                  <a:lumMod val="95000"/>
+                </a:schemeClr>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>B1</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>730250</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>120649</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>321733</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>4232</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="8" name="TextBox 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{45CE4122-5C27-F34E-94F9-0ECC70C48405}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="12020550" y="1454149"/>
+          <a:ext cx="416983" cy="264583"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525" cmpd="sng">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="bg1">
+                  <a:lumMod val="95000"/>
+                </a:schemeClr>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>B12</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>74083</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>27516</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>410633</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>101599</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="9" name="TextBox 8">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{AAB33BA8-1451-9C41-BA86-CC93E9F96D65}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6411383" y="5742516"/>
+          <a:ext cx="336550" cy="264583"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525" cmpd="sng">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="bg1">
+                  <a:lumMod val="95000"/>
+                </a:schemeClr>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>C2</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>402167</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>154517</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>751417</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="10" name="TextBox 9">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DDC6A946-D838-6842-A2F8-B7DD889821AF}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="10041467" y="5679017"/>
+          <a:ext cx="349250" cy="264583"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525" cmpd="sng">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="bg1">
+                  <a:lumMod val="95000"/>
+                </a:schemeClr>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>D4</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>702733</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>148167</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>226483</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>31750</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="11" name="TextBox 10">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FB293869-091C-D349-8ECA-02D30EF04AFB}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="10342033" y="5672667"/>
+          <a:ext cx="349250" cy="264583"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525" cmpd="sng">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="bg1">
+                  <a:lumMod val="95000"/>
+                </a:schemeClr>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>D5</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>31750</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>154517</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>381000</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="12" name="TextBox 11">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E1E27EE9-4004-1242-8AB9-FAA16B637321}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="11322050" y="5679017"/>
+          <a:ext cx="349250" cy="264583"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525" cmpd="sng">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="bg1">
+                  <a:lumMod val="95000"/>
+                </a:schemeClr>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>D9</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>321734</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>158750</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>740834</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>42333</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="13" name="TextBox 12">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5D2485E3-AF19-5444-84BE-3836298BD313}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="11612034" y="5683250"/>
+          <a:ext cx="419100" cy="264583"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525" cmpd="sng">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="bg1">
+                  <a:lumMod val="95000"/>
+                </a:schemeClr>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>D10</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>469900</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>95250</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>819150</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>169333</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="15" name="TextBox 14">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{020600C1-4C98-0542-8757-7C470439398C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="13411200" y="1619250"/>
+          <a:ext cx="349250" cy="264583"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525" cmpd="sng">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>E4</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>357717</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>184150</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>706967</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>67733</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="16" name="TextBox 15">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C2B48461-002E-B945-9B7F-BFF384B2DEB1}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="13299017" y="5518150"/>
+          <a:ext cx="349250" cy="264583"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525" cmpd="sng">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>E5</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>353484</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>150282</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>768350</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>33865</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="17" name="TextBox 16">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F7F451F3-8987-004C-A4C8-9E65B0BEB285}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="8341784" y="1483782"/>
+          <a:ext cx="414866" cy="264583"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525" cmpd="sng">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="bg1">
+                  <a:lumMod val="95000"/>
+                </a:schemeClr>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>A10</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>124884</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>150282</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>539750</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>33865</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="18" name="TextBox 17">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A91C5B34-8140-6F40-BEE8-C1AE81F15D67}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="8113184" y="1483782"/>
+          <a:ext cx="414866" cy="264583"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525" cmpd="sng">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="bg1">
+                  <a:lumMod val="95000"/>
+                </a:schemeClr>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>A9</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
@@ -2764,70 +3928,70 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="48" t="s">
+      <c r="A1" s="55" t="s">
         <v>71</v>
       </c>
-      <c r="B1" s="48"/>
-      <c r="C1" s="48"/>
-      <c r="D1" s="48"/>
-      <c r="E1" s="48"/>
-      <c r="F1" s="48"/>
-      <c r="G1" s="48"/>
-      <c r="H1" s="48"/>
-      <c r="I1" s="48"/>
-      <c r="J1" s="48"/>
-      <c r="K1" s="48"/>
-      <c r="L1" s="48"/>
-      <c r="M1" s="48"/>
-      <c r="N1" s="48"/>
+      <c r="B1" s="55"/>
+      <c r="C1" s="55"/>
+      <c r="D1" s="55"/>
+      <c r="E1" s="55"/>
+      <c r="F1" s="55"/>
+      <c r="G1" s="55"/>
+      <c r="H1" s="55"/>
+      <c r="I1" s="55"/>
+      <c r="J1" s="55"/>
+      <c r="K1" s="55"/>
+      <c r="L1" s="55"/>
+      <c r="M1" s="55"/>
+      <c r="N1" s="55"/>
     </row>
     <row r="2" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="48"/>
-      <c r="B2" s="48"/>
-      <c r="C2" s="48"/>
-      <c r="D2" s="48"/>
-      <c r="E2" s="48"/>
-      <c r="F2" s="48"/>
-      <c r="G2" s="48"/>
-      <c r="H2" s="48"/>
-      <c r="I2" s="48"/>
-      <c r="J2" s="48"/>
-      <c r="K2" s="48"/>
-      <c r="L2" s="48"/>
-      <c r="M2" s="48"/>
-      <c r="N2" s="48"/>
+      <c r="A2" s="55"/>
+      <c r="B2" s="55"/>
+      <c r="C2" s="55"/>
+      <c r="D2" s="55"/>
+      <c r="E2" s="55"/>
+      <c r="F2" s="55"/>
+      <c r="G2" s="55"/>
+      <c r="H2" s="55"/>
+      <c r="I2" s="55"/>
+      <c r="J2" s="55"/>
+      <c r="K2" s="55"/>
+      <c r="L2" s="55"/>
+      <c r="M2" s="55"/>
+      <c r="N2" s="55"/>
     </row>
     <row r="3" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="48"/>
-      <c r="B3" s="48"/>
-      <c r="C3" s="48"/>
-      <c r="D3" s="48"/>
-      <c r="E3" s="48"/>
-      <c r="F3" s="48"/>
-      <c r="G3" s="48"/>
-      <c r="H3" s="48"/>
-      <c r="I3" s="48"/>
-      <c r="J3" s="48"/>
-      <c r="K3" s="48"/>
-      <c r="L3" s="48"/>
-      <c r="M3" s="48"/>
-      <c r="N3" s="48"/>
+      <c r="A3" s="55"/>
+      <c r="B3" s="55"/>
+      <c r="C3" s="55"/>
+      <c r="D3" s="55"/>
+      <c r="E3" s="55"/>
+      <c r="F3" s="55"/>
+      <c r="G3" s="55"/>
+      <c r="H3" s="55"/>
+      <c r="I3" s="55"/>
+      <c r="J3" s="55"/>
+      <c r="K3" s="55"/>
+      <c r="L3" s="55"/>
+      <c r="M3" s="55"/>
+      <c r="N3" s="55"/>
     </row>
     <row r="4" spans="1:17" ht="21" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="48"/>
-      <c r="B4" s="48"/>
-      <c r="C4" s="48"/>
-      <c r="D4" s="48"/>
-      <c r="E4" s="48"/>
-      <c r="F4" s="48"/>
-      <c r="G4" s="48"/>
-      <c r="H4" s="48"/>
-      <c r="I4" s="48"/>
-      <c r="J4" s="48"/>
-      <c r="K4" s="48"/>
-      <c r="L4" s="48"/>
-      <c r="M4" s="48"/>
-      <c r="N4" s="48"/>
+      <c r="A4" s="55"/>
+      <c r="B4" s="55"/>
+      <c r="C4" s="55"/>
+      <c r="D4" s="55"/>
+      <c r="E4" s="55"/>
+      <c r="F4" s="55"/>
+      <c r="G4" s="55"/>
+      <c r="H4" s="55"/>
+      <c r="I4" s="55"/>
+      <c r="J4" s="55"/>
+      <c r="K4" s="55"/>
+      <c r="L4" s="55"/>
+      <c r="M4" s="55"/>
+      <c r="N4" s="55"/>
     </row>
     <row r="5" spans="1:17" ht="21" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="17"/>
@@ -4554,51 +5718,51 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A1" s="48" t="s">
+      <c r="A1" s="55" t="s">
         <v>611</v>
       </c>
-      <c r="B1" s="48"/>
-      <c r="C1" s="48"/>
-      <c r="D1" s="48"/>
-      <c r="E1" s="48"/>
-      <c r="F1" s="48"/>
-      <c r="G1" s="48"/>
-      <c r="H1" s="48"/>
-      <c r="I1" s="48"/>
-      <c r="J1" s="48"/>
-      <c r="K1" s="48"/>
-      <c r="L1" s="48"/>
-      <c r="M1" s="48"/>
+      <c r="B1" s="55"/>
+      <c r="C1" s="55"/>
+      <c r="D1" s="55"/>
+      <c r="E1" s="55"/>
+      <c r="F1" s="55"/>
+      <c r="G1" s="55"/>
+      <c r="H1" s="55"/>
+      <c r="I1" s="55"/>
+      <c r="J1" s="55"/>
+      <c r="K1" s="55"/>
+      <c r="L1" s="55"/>
+      <c r="M1" s="55"/>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A2" s="48"/>
-      <c r="B2" s="48"/>
-      <c r="C2" s="48"/>
-      <c r="D2" s="48"/>
-      <c r="E2" s="48"/>
-      <c r="F2" s="48"/>
-      <c r="G2" s="48"/>
-      <c r="H2" s="48"/>
-      <c r="I2" s="48"/>
-      <c r="J2" s="48"/>
-      <c r="K2" s="48"/>
-      <c r="L2" s="48"/>
-      <c r="M2" s="48"/>
+      <c r="A2" s="55"/>
+      <c r="B2" s="55"/>
+      <c r="C2" s="55"/>
+      <c r="D2" s="55"/>
+      <c r="E2" s="55"/>
+      <c r="F2" s="55"/>
+      <c r="G2" s="55"/>
+      <c r="H2" s="55"/>
+      <c r="I2" s="55"/>
+      <c r="J2" s="55"/>
+      <c r="K2" s="55"/>
+      <c r="L2" s="55"/>
+      <c r="M2" s="55"/>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A3" s="48"/>
-      <c r="B3" s="48"/>
-      <c r="C3" s="48"/>
-      <c r="D3" s="48"/>
-      <c r="E3" s="48"/>
-      <c r="F3" s="48"/>
-      <c r="G3" s="48"/>
-      <c r="H3" s="48"/>
-      <c r="I3" s="48"/>
-      <c r="J3" s="48"/>
-      <c r="K3" s="48"/>
-      <c r="L3" s="48"/>
-      <c r="M3" s="48"/>
+      <c r="A3" s="55"/>
+      <c r="B3" s="55"/>
+      <c r="C3" s="55"/>
+      <c r="D3" s="55"/>
+      <c r="E3" s="55"/>
+      <c r="F3" s="55"/>
+      <c r="G3" s="55"/>
+      <c r="H3" s="55"/>
+      <c r="I3" s="55"/>
+      <c r="J3" s="55"/>
+      <c r="K3" s="55"/>
+      <c r="L3" s="55"/>
+      <c r="M3" s="55"/>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A6" s="13"/>
@@ -4643,40 +5807,40 @@
       <c r="A7" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="B7" s="49" t="s">
+      <c r="B7" s="25" t="s">
         <v>73</v>
       </c>
-      <c r="C7" s="49" t="s">
+      <c r="C7" s="25" t="s">
         <v>74</v>
       </c>
-      <c r="D7" s="50" t="s">
+      <c r="D7" s="48" t="s">
         <v>88</v>
       </c>
-      <c r="E7" s="49" t="s">
+      <c r="E7" s="25" t="s">
         <v>89</v>
       </c>
-      <c r="F7" s="50" t="s">
+      <c r="F7" s="48" t="s">
         <v>90</v>
       </c>
-      <c r="G7" s="49" t="s">
+      <c r="G7" s="25" t="s">
         <v>88</v>
       </c>
-      <c r="H7" s="49" t="s">
+      <c r="H7" s="25" t="s">
         <v>100</v>
       </c>
-      <c r="I7" s="49" t="s">
+      <c r="I7" s="25" t="s">
         <v>93</v>
       </c>
-      <c r="J7" s="50" t="s">
+      <c r="J7" s="48" t="s">
         <v>101</v>
       </c>
-      <c r="K7" s="50" t="s">
+      <c r="K7" s="48" t="s">
         <v>95</v>
       </c>
-      <c r="L7" s="50" t="s">
+      <c r="L7" s="48" t="s">
         <v>93</v>
       </c>
-      <c r="M7" s="49"/>
+      <c r="M7" s="25"/>
       <c r="N7" t="s">
         <v>72</v>
       </c>
@@ -4694,40 +5858,40 @@
       <c r="A8" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="B8" s="50" t="s">
+      <c r="B8" s="48" t="s">
         <v>76</v>
       </c>
-      <c r="C8" s="49" t="s">
+      <c r="C8" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="D8" s="50" t="s">
+      <c r="D8" s="48" t="s">
         <v>78</v>
       </c>
-      <c r="E8" s="49" t="s">
+      <c r="E8" s="25" t="s">
         <v>79</v>
       </c>
-      <c r="F8" s="49" t="s">
+      <c r="F8" s="25" t="s">
         <v>80</v>
       </c>
-      <c r="G8" s="49" t="s">
+      <c r="G8" s="25" t="s">
         <v>81</v>
       </c>
-      <c r="H8" s="49" t="s">
+      <c r="H8" s="25" t="s">
         <v>103</v>
       </c>
-      <c r="I8" s="49" t="s">
+      <c r="I8" s="25" t="s">
         <v>431</v>
       </c>
-      <c r="J8" s="49" t="s">
+      <c r="J8" s="25" t="s">
         <v>83</v>
       </c>
-      <c r="K8" s="49" t="s">
+      <c r="K8" s="25" t="s">
         <v>84</v>
       </c>
-      <c r="L8" s="49" t="s">
+      <c r="L8" s="25" t="s">
         <v>85</v>
       </c>
-      <c r="M8" s="50" t="s">
+      <c r="M8" s="48" t="s">
         <v>86</v>
       </c>
       <c r="N8" t="s">
@@ -4738,40 +5902,40 @@
       <c r="A9" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="B9" s="49" t="s">
+      <c r="B9" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="C9" s="50" t="s">
+      <c r="C9" s="48" t="s">
         <v>92</v>
       </c>
-      <c r="D9" s="49" t="s">
+      <c r="D9" s="25" t="s">
         <v>93</v>
       </c>
-      <c r="E9" s="49" t="s">
+      <c r="E9" s="25" t="s">
         <v>94</v>
       </c>
-      <c r="F9" s="49" t="s">
+      <c r="F9" s="25" t="s">
         <v>95</v>
       </c>
-      <c r="G9" s="50" t="s">
+      <c r="G9" s="48" t="s">
         <v>96</v>
       </c>
-      <c r="H9" s="50" t="s">
+      <c r="H9" s="48" t="s">
         <v>97</v>
       </c>
-      <c r="I9" s="50" t="s">
+      <c r="I9" s="48" t="s">
         <v>84</v>
       </c>
-      <c r="J9" s="49" t="s">
+      <c r="J9" s="25" t="s">
         <v>85</v>
       </c>
-      <c r="K9" s="49" t="s">
+      <c r="K9" s="25" t="s">
         <v>108</v>
       </c>
-      <c r="L9" s="50" t="s">
+      <c r="L9" s="48" t="s">
         <v>109</v>
       </c>
-      <c r="M9" s="49" t="s">
+      <c r="M9" s="25" t="s">
         <v>110</v>
       </c>
       <c r="N9" t="s">
@@ -4785,40 +5949,40 @@
       <c r="A10" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="B10" s="49" t="s">
+      <c r="B10" s="25" t="s">
         <v>100</v>
       </c>
-      <c r="C10" s="50" t="s">
+      <c r="C10" s="48" t="s">
         <v>81</v>
       </c>
-      <c r="D10" s="49" t="s">
+      <c r="D10" s="25" t="s">
         <v>103</v>
       </c>
-      <c r="E10" s="50" t="s">
+      <c r="E10" s="48" t="s">
         <v>93</v>
       </c>
-      <c r="F10" s="50" t="s">
+      <c r="F10" s="48" t="s">
         <v>104</v>
       </c>
-      <c r="G10" s="49" t="s">
+      <c r="G10" s="25" t="s">
         <v>105</v>
       </c>
-      <c r="H10" s="49" t="s">
+      <c r="H10" s="25" t="s">
         <v>94</v>
       </c>
-      <c r="I10" s="49" t="s">
+      <c r="I10" s="25" t="s">
         <v>106</v>
       </c>
-      <c r="J10" s="50" t="s">
+      <c r="J10" s="48" t="s">
         <v>113</v>
       </c>
-      <c r="K10" s="50" t="s">
+      <c r="K10" s="48" t="s">
         <v>104</v>
       </c>
-      <c r="L10" s="50" t="s">
+      <c r="L10" s="48" t="s">
         <v>114</v>
       </c>
-      <c r="M10" s="49"/>
+      <c r="M10" s="25"/>
       <c r="N10" t="s">
         <v>102</v>
       </c>
@@ -4830,30 +5994,30 @@
       <c r="A11" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="B11" s="49" t="s">
+      <c r="B11" s="25" t="s">
         <v>116</v>
       </c>
-      <c r="C11" s="49" t="s">
+      <c r="C11" s="25" t="s">
         <v>118</v>
       </c>
-      <c r="D11" s="49" t="s">
+      <c r="D11" s="25" t="s">
         <v>117</v>
       </c>
-      <c r="E11" s="50" t="s">
+      <c r="E11" s="48" t="s">
         <v>95</v>
       </c>
-      <c r="F11" s="50" t="s">
+      <c r="F11" s="48" t="s">
         <v>106</v>
       </c>
-      <c r="G11" s="49" t="s">
+      <c r="G11" s="25" t="s">
         <v>119</v>
       </c>
-      <c r="H11" s="49"/>
-      <c r="I11" s="49"/>
-      <c r="J11" s="49"/>
-      <c r="K11" s="49"/>
-      <c r="L11" s="49"/>
-      <c r="M11" s="49"/>
+      <c r="H11" s="25"/>
+      <c r="I11" s="25"/>
+      <c r="J11" s="25"/>
+      <c r="K11" s="25"/>
+      <c r="L11" s="25"/>
+      <c r="M11" s="25"/>
       <c r="N11" t="s">
         <v>115</v>
       </c>
@@ -4862,55 +6026,55 @@
       <c r="A12" s="13" t="s">
         <v>29</v>
       </c>
-      <c r="B12" s="49"/>
-      <c r="C12" s="49"/>
-      <c r="D12" s="49"/>
-      <c r="E12" s="49"/>
-      <c r="F12" s="49"/>
-      <c r="G12" s="49"/>
-      <c r="H12" s="49"/>
-      <c r="I12" s="49"/>
-      <c r="J12" s="49"/>
-      <c r="K12" s="49"/>
-      <c r="L12" s="49"/>
-      <c r="M12" s="49"/>
+      <c r="B12" s="25"/>
+      <c r="C12" s="25"/>
+      <c r="D12" s="25"/>
+      <c r="E12" s="25"/>
+      <c r="F12" s="25"/>
+      <c r="G12" s="25"/>
+      <c r="H12" s="25"/>
+      <c r="I12" s="25"/>
+      <c r="J12" s="25"/>
+      <c r="K12" s="25"/>
+      <c r="L12" s="25"/>
+      <c r="M12" s="25"/>
     </row>
     <row r="13" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A13" s="13" t="s">
         <v>30</v>
       </c>
-      <c r="B13" s="49"/>
-      <c r="C13" s="49"/>
-      <c r="D13" s="49"/>
-      <c r="E13" s="49"/>
-      <c r="F13" s="49"/>
-      <c r="G13" s="49"/>
-      <c r="H13" s="49"/>
-      <c r="I13" s="49"/>
-      <c r="J13" s="49"/>
-      <c r="K13" s="49"/>
-      <c r="L13" s="49"/>
-      <c r="M13" s="49"/>
+      <c r="B13" s="25"/>
+      <c r="C13" s="25"/>
+      <c r="D13" s="25"/>
+      <c r="E13" s="25"/>
+      <c r="F13" s="25"/>
+      <c r="G13" s="25"/>
+      <c r="H13" s="25"/>
+      <c r="I13" s="25"/>
+      <c r="J13" s="25"/>
+      <c r="K13" s="25"/>
+      <c r="L13" s="25"/>
+      <c r="M13" s="25"/>
     </row>
     <row r="14" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A14" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="B14" s="49"/>
-      <c r="C14" s="49"/>
-      <c r="D14" s="49"/>
-      <c r="E14" s="49"/>
-      <c r="F14" s="49"/>
-      <c r="G14" s="49"/>
-      <c r="H14" s="49"/>
-      <c r="I14" s="49"/>
-      <c r="J14" s="49"/>
-      <c r="K14" s="49"/>
-      <c r="L14" s="49"/>
-      <c r="M14" s="49"/>
+      <c r="B14" s="25"/>
+      <c r="C14" s="25"/>
+      <c r="D14" s="25"/>
+      <c r="E14" s="25"/>
+      <c r="F14" s="25"/>
+      <c r="G14" s="25"/>
+      <c r="H14" s="25"/>
+      <c r="I14" s="25"/>
+      <c r="J14" s="25"/>
+      <c r="K14" s="25"/>
+      <c r="L14" s="25"/>
+      <c r="M14" s="25"/>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A17" s="51"/>
+      <c r="A17" s="13"/>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.2">
       <c r="B18" t="s">
@@ -4952,7 +6116,7 @@
     </row>
     <row r="21" spans="1:13" ht="16" x14ac:dyDescent="0.2">
       <c r="A21" s="1"/>
-      <c r="B21" s="52" t="s">
+      <c r="B21" s="49" t="s">
         <v>590</v>
       </c>
       <c r="C21" s="6">
@@ -4962,7 +6126,7 @@
         <f>D19*C21*1.05</f>
         <v>288.75</v>
       </c>
-      <c r="G21" s="52" t="s">
+      <c r="G21" s="49" t="s">
         <v>590</v>
       </c>
       <c r="H21" s="6">
@@ -4975,7 +6139,7 @@
     </row>
     <row r="22" spans="1:13" ht="16" x14ac:dyDescent="0.2">
       <c r="A22" s="1"/>
-      <c r="B22" s="52" t="s">
+      <c r="B22" s="49" t="s">
         <v>593</v>
       </c>
       <c r="C22" s="6">
@@ -4985,7 +6149,7 @@
         <f>D19*C22*1.05</f>
         <v>28.875</v>
       </c>
-      <c r="G22" s="52" t="s">
+      <c r="G22" s="49" t="s">
         <v>593</v>
       </c>
       <c r="H22" s="6">
@@ -4998,7 +6162,7 @@
     </row>
     <row r="23" spans="1:13" ht="16" x14ac:dyDescent="0.2">
       <c r="A23" s="1"/>
-      <c r="B23" s="52" t="s">
+      <c r="B23" s="49" t="s">
         <v>594</v>
       </c>
       <c r="C23" s="6">
@@ -5008,7 +6172,7 @@
         <f>D19*C23*1.05</f>
         <v>28.875</v>
       </c>
-      <c r="G23" s="52" t="s">
+      <c r="G23" s="49" t="s">
         <v>595</v>
       </c>
       <c r="H23" s="6">
@@ -5021,7 +6185,7 @@
     </row>
     <row r="24" spans="1:13" ht="16" x14ac:dyDescent="0.2">
       <c r="A24" s="1"/>
-      <c r="B24" s="52" t="s">
+      <c r="B24" s="49" t="s">
         <v>591</v>
       </c>
       <c r="C24" s="6">
@@ -5031,7 +6195,7 @@
         <f>D19*C24*1.05</f>
         <v>115.5</v>
       </c>
-      <c r="G24" s="52" t="s">
+      <c r="G24" s="49" t="s">
         <v>591</v>
       </c>
       <c r="H24" s="6">
@@ -5198,25 +6362,25 @@
       <c r="K30" s="27" t="s">
         <v>592</v>
       </c>
-      <c r="L30" s="49"/>
-      <c r="M30" s="49"/>
+      <c r="L30" s="25"/>
+      <c r="M30" s="25"/>
     </row>
     <row r="31" spans="1:13" ht="16" x14ac:dyDescent="0.2">
       <c r="A31" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="B31" s="49"/>
-      <c r="C31" s="49"/>
-      <c r="D31" s="49"/>
-      <c r="E31" s="49"/>
-      <c r="F31" s="49"/>
-      <c r="G31" s="49"/>
-      <c r="H31" s="49"/>
-      <c r="I31" s="49"/>
-      <c r="J31" s="49"/>
-      <c r="K31" s="49"/>
-      <c r="L31" s="49"/>
-      <c r="M31" s="49"/>
+      <c r="B31" s="25"/>
+      <c r="C31" s="25"/>
+      <c r="D31" s="25"/>
+      <c r="E31" s="25"/>
+      <c r="F31" s="25"/>
+      <c r="G31" s="25"/>
+      <c r="H31" s="25"/>
+      <c r="I31" s="25"/>
+      <c r="J31" s="25"/>
+      <c r="K31" s="25"/>
+      <c r="L31" s="25"/>
+      <c r="M31" s="25"/>
     </row>
     <row r="32" spans="1:13" ht="16" x14ac:dyDescent="0.2">
       <c r="A32" s="13" t="s">
@@ -5293,154 +6457,154 @@
       <c r="K33" s="28" t="s">
         <v>592</v>
       </c>
-      <c r="L33" s="49"/>
-      <c r="M33" s="49"/>
+      <c r="L33" s="25"/>
+      <c r="M33" s="25"/>
     </row>
     <row r="34" spans="1:13" ht="16" x14ac:dyDescent="0.2">
       <c r="A34" s="13" t="s">
         <v>29</v>
       </c>
-      <c r="B34" s="49"/>
-      <c r="C34" s="49"/>
-      <c r="D34" s="49"/>
-      <c r="E34" s="49"/>
-      <c r="F34" s="49"/>
-      <c r="G34" s="49"/>
-      <c r="H34" s="49"/>
-      <c r="I34" s="49"/>
-      <c r="J34" s="49"/>
-      <c r="K34" s="49"/>
-      <c r="L34" s="49"/>
-      <c r="M34" s="49"/>
+      <c r="B34" s="25"/>
+      <c r="C34" s="25"/>
+      <c r="D34" s="25"/>
+      <c r="E34" s="25"/>
+      <c r="F34" s="25"/>
+      <c r="G34" s="25"/>
+      <c r="H34" s="25"/>
+      <c r="I34" s="25"/>
+      <c r="J34" s="25"/>
+      <c r="K34" s="25"/>
+      <c r="L34" s="25"/>
+      <c r="M34" s="25"/>
     </row>
     <row r="35" spans="1:13" ht="16" x14ac:dyDescent="0.2">
       <c r="A35" s="13" t="s">
         <v>30</v>
       </c>
-      <c r="B35" s="49"/>
-      <c r="C35" s="49"/>
-      <c r="D35" s="49"/>
-      <c r="E35" s="49"/>
-      <c r="F35" s="49"/>
-      <c r="G35" s="49"/>
-      <c r="H35" s="49"/>
-      <c r="I35" s="49"/>
-      <c r="J35" s="49"/>
-      <c r="K35" s="49"/>
-      <c r="L35" s="49"/>
-      <c r="M35" s="49"/>
+      <c r="B35" s="25"/>
+      <c r="C35" s="25"/>
+      <c r="D35" s="25"/>
+      <c r="E35" s="25"/>
+      <c r="F35" s="25"/>
+      <c r="G35" s="25"/>
+      <c r="H35" s="25"/>
+      <c r="I35" s="25"/>
+      <c r="J35" s="25"/>
+      <c r="K35" s="25"/>
+      <c r="L35" s="25"/>
+      <c r="M35" s="25"/>
     </row>
     <row r="36" spans="1:13" ht="16" x14ac:dyDescent="0.2">
       <c r="A36" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="B36" s="49"/>
-      <c r="C36" s="49"/>
-      <c r="D36" s="49"/>
-      <c r="E36" s="49"/>
-      <c r="F36" s="49"/>
-      <c r="G36" s="49"/>
-      <c r="H36" s="49"/>
-      <c r="I36" s="49"/>
-      <c r="J36" s="49"/>
-      <c r="K36" s="49"/>
-      <c r="L36" s="49"/>
-      <c r="M36" s="49"/>
+      <c r="B36" s="25"/>
+      <c r="C36" s="25"/>
+      <c r="D36" s="25"/>
+      <c r="E36" s="25"/>
+      <c r="F36" s="25"/>
+      <c r="G36" s="25"/>
+      <c r="H36" s="25"/>
+      <c r="I36" s="25"/>
+      <c r="J36" s="25"/>
+      <c r="K36" s="25"/>
+      <c r="L36" s="25"/>
+      <c r="M36" s="25"/>
     </row>
     <row r="39" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A39" s="53" t="s">
+      <c r="A39" s="50" t="s">
         <v>597</v>
       </c>
     </row>
     <row r="40" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="B40" s="54" t="s">
+      <c r="B40" s="51" t="s">
         <v>598</v>
       </c>
-      <c r="C40" s="54" t="s">
+      <c r="C40" s="51" t="s">
         <v>599</v>
       </c>
-      <c r="D40" s="54" t="s">
+      <c r="D40" s="51" t="s">
         <v>600</v>
       </c>
-      <c r="E40" s="56" t="s">
+      <c r="E40" t="s">
         <v>607</v>
       </c>
     </row>
     <row r="41" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="B41" s="55" t="s">
+      <c r="B41" s="52" t="s">
         <v>603</v>
       </c>
-      <c r="C41" s="55">
+      <c r="C41" s="52">
         <v>98</v>
       </c>
-      <c r="D41" s="55" t="s">
+      <c r="D41" s="52" t="s">
         <v>18</v>
       </c>
-      <c r="E41" s="57">
+      <c r="E41" s="53">
         <v>1</v>
       </c>
     </row>
     <row r="42" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="B42" s="55" t="s">
+      <c r="B42" s="52" t="s">
         <v>604</v>
       </c>
-      <c r="C42" s="55">
+      <c r="C42" s="52">
         <v>98</v>
       </c>
-      <c r="D42" s="55" t="s">
+      <c r="D42" s="52" t="s">
         <v>608</v>
       </c>
-      <c r="E42" s="58">
+      <c r="E42" s="56">
         <v>30</v>
       </c>
     </row>
     <row r="43" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="B43" s="55" t="s">
+      <c r="B43" s="52" t="s">
         <v>605</v>
       </c>
-      <c r="C43" s="55">
+      <c r="C43" s="52">
         <v>65</v>
       </c>
-      <c r="D43" s="55" t="s">
+      <c r="D43" s="52" t="s">
         <v>609</v>
       </c>
-      <c r="E43" s="59"/>
+      <c r="E43" s="57"/>
     </row>
     <row r="44" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="B44" s="55" t="s">
+      <c r="B44" s="52" t="s">
         <v>606</v>
       </c>
-      <c r="C44" s="55">
+      <c r="C44" s="52">
         <v>72</v>
       </c>
-      <c r="D44" s="55" t="s">
+      <c r="D44" s="52" t="s">
         <v>609</v>
       </c>
-      <c r="E44" s="60"/>
+      <c r="E44" s="58"/>
     </row>
     <row r="45" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="B45" s="55" t="s">
+      <c r="B45" s="52" t="s">
         <v>610</v>
       </c>
-      <c r="C45" s="55">
+      <c r="C45" s="52">
         <v>72</v>
       </c>
-      <c r="D45" s="55" t="s">
+      <c r="D45" s="52" t="s">
         <v>601</v>
       </c>
-      <c r="E45" s="61">
+      <c r="E45" s="54">
         <v>1</v>
       </c>
     </row>
     <row r="46" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="B46" s="55" t="s">
+      <c r="B46" s="52" t="s">
         <v>602</v>
       </c>
-      <c r="C46" s="55">
+      <c r="C46" s="52">
         <v>4</v>
       </c>
-      <c r="D46" s="55"/>
-      <c r="E46" s="57"/>
+      <c r="D46" s="52"/>
+      <c r="E46" s="53"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -9238,4 +10402,352 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="25" fitToHeight="3" orientation="landscape" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D63679B-89D8-7444-9872-85CD4FFE082B}">
+  <dimension ref="A1:G15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="12" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.5" customWidth="1"/>
+    <col min="4" max="4" width="70.83203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.83203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A1" s="59" t="s">
+        <v>612</v>
+      </c>
+      <c r="B1" s="59" t="s">
+        <v>613</v>
+      </c>
+      <c r="C1" s="59" t="s">
+        <v>628</v>
+      </c>
+      <c r="D1" s="59" t="s">
+        <v>632</v>
+      </c>
+      <c r="E1" s="59" t="s">
+        <v>634</v>
+      </c>
+      <c r="F1" s="59" t="s">
+        <v>642</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A2" s="59" t="s">
+        <v>614</v>
+      </c>
+      <c r="B2" s="59" t="s">
+        <v>88</v>
+      </c>
+      <c r="C2" s="59" t="s">
+        <v>629</v>
+      </c>
+      <c r="D2" s="61" t="s">
+        <v>633</v>
+      </c>
+      <c r="E2" s="61" t="s">
+        <v>635</v>
+      </c>
+      <c r="F2" s="61">
+        <v>93.68</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A3" s="59" t="s">
+        <v>615</v>
+      </c>
+      <c r="B3" s="59" t="s">
+        <v>528</v>
+      </c>
+      <c r="C3" s="59" t="s">
+        <v>629</v>
+      </c>
+      <c r="D3" s="61" t="s">
+        <v>633</v>
+      </c>
+      <c r="E3" s="61" t="s">
+        <v>635</v>
+      </c>
+      <c r="F3" s="61">
+        <v>93.56</v>
+      </c>
+      <c r="G3" s="60"/>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A4" s="59" t="s">
+        <v>622</v>
+      </c>
+      <c r="B4" s="59" t="s">
+        <v>108</v>
+      </c>
+      <c r="C4" s="59" t="s">
+        <v>630</v>
+      </c>
+      <c r="D4" s="61" t="s">
+        <v>633</v>
+      </c>
+      <c r="E4" s="61" t="s">
+        <v>635</v>
+      </c>
+      <c r="F4" s="61">
+        <v>88.37</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" s="66" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="64" t="s">
+        <v>623</v>
+      </c>
+      <c r="B5" s="64" t="s">
+        <v>530</v>
+      </c>
+      <c r="C5" s="64" t="s">
+        <v>631</v>
+      </c>
+      <c r="D5" s="61" t="s">
+        <v>638</v>
+      </c>
+      <c r="E5" s="61" t="s">
+        <v>639</v>
+      </c>
+      <c r="F5" s="65">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A6" s="59" t="s">
+        <v>617</v>
+      </c>
+      <c r="B6" s="59" t="s">
+        <v>539</v>
+      </c>
+      <c r="C6" s="59" t="s">
+        <v>630</v>
+      </c>
+      <c r="D6" s="61" t="s">
+        <v>633</v>
+      </c>
+      <c r="E6" s="61" t="s">
+        <v>635</v>
+      </c>
+      <c r="F6" s="61">
+        <v>93.6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A7" s="59" t="s">
+        <v>624</v>
+      </c>
+      <c r="B7" s="59" t="s">
+        <v>76</v>
+      </c>
+      <c r="C7" s="59" t="s">
+        <v>630</v>
+      </c>
+      <c r="D7" s="61" t="s">
+        <v>633</v>
+      </c>
+      <c r="E7" s="61" t="s">
+        <v>635</v>
+      </c>
+      <c r="F7" s="61">
+        <v>91.53</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A8" s="59" t="s">
+        <v>625</v>
+      </c>
+      <c r="B8" s="59" t="s">
+        <v>539</v>
+      </c>
+      <c r="C8" s="59" t="s">
+        <v>631</v>
+      </c>
+      <c r="D8" s="61" t="s">
+        <v>643</v>
+      </c>
+      <c r="E8" s="61" t="s">
+        <v>644</v>
+      </c>
+      <c r="F8" s="61" t="s">
+        <v>644</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A9" s="62" t="s">
+        <v>616</v>
+      </c>
+      <c r="B9" s="62" t="s">
+        <v>540</v>
+      </c>
+      <c r="C9" s="62" t="s">
+        <v>629</v>
+      </c>
+      <c r="D9" s="63" t="s">
+        <v>637</v>
+      </c>
+      <c r="E9" s="63" t="s">
+        <v>636</v>
+      </c>
+      <c r="F9" s="63">
+        <v>99.27</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A10" s="59" t="s">
+        <v>626</v>
+      </c>
+      <c r="B10" s="59" t="s">
+        <v>79</v>
+      </c>
+      <c r="C10" s="59" t="s">
+        <v>631</v>
+      </c>
+      <c r="D10" s="61" t="s">
+        <v>633</v>
+      </c>
+      <c r="E10" s="61" t="s">
+        <v>635</v>
+      </c>
+      <c r="F10" s="61">
+        <v>93.63</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A11" s="59" t="s">
+        <v>627</v>
+      </c>
+      <c r="B11" s="59" t="s">
+        <v>550</v>
+      </c>
+      <c r="C11" s="59" t="s">
+        <v>630</v>
+      </c>
+      <c r="D11" s="61" t="s">
+        <v>633</v>
+      </c>
+      <c r="E11" s="61" t="s">
+        <v>635</v>
+      </c>
+      <c r="F11" s="61">
+        <v>92.9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A12" s="59" t="s">
+        <v>618</v>
+      </c>
+      <c r="B12" s="59" t="s">
+        <v>117</v>
+      </c>
+      <c r="C12" s="59" t="s">
+        <v>631</v>
+      </c>
+      <c r="D12" s="61" t="s">
+        <v>633</v>
+      </c>
+      <c r="E12" s="61" t="s">
+        <v>635</v>
+      </c>
+      <c r="F12" s="61">
+        <v>93.63</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A13" s="59" t="s">
+        <v>619</v>
+      </c>
+      <c r="B13" s="59" t="s">
+        <v>80</v>
+      </c>
+      <c r="C13" s="59" t="s">
+        <v>629</v>
+      </c>
+      <c r="D13" s="61" t="s">
+        <v>633</v>
+      </c>
+      <c r="E13" s="61" t="s">
+        <v>635</v>
+      </c>
+      <c r="F13" s="61">
+        <v>93.8</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A14" s="59" t="s">
+        <v>620</v>
+      </c>
+      <c r="B14" s="59" t="s">
+        <v>93</v>
+      </c>
+      <c r="C14" s="59" t="s">
+        <v>630</v>
+      </c>
+      <c r="D14" s="61" t="s">
+        <v>633</v>
+      </c>
+      <c r="E14" s="61" t="s">
+        <v>635</v>
+      </c>
+      <c r="F14" s="61">
+        <v>93.24</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A15" s="62" t="s">
+        <v>621</v>
+      </c>
+      <c r="B15" s="62" t="s">
+        <v>104</v>
+      </c>
+      <c r="C15" s="62" t="s">
+        <v>629</v>
+      </c>
+      <c r="D15" s="63" t="s">
+        <v>640</v>
+      </c>
+      <c r="E15" s="63" t="s">
+        <v>641</v>
+      </c>
+      <c r="F15" s="63">
+        <v>100</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="D3" r:id="rId1" location="alnHdr_18030094" tooltip="Go to alignment for Drosophila melanogaster X BAC RP98-12H1 (Roswell Park Cancer Institute Drosophila BAC Library) complete sequence" display="https://blast.ncbi.nlm.nih.gov/Blast.cgi - alnHdr_18030094" xr:uid="{F4989C41-D768-8046-A42B-A93241C11AF0}"/>
+    <hyperlink ref="E3" r:id="rId2" tooltip="Show report for AC023691.3" display="https://www.ncbi.nlm.nih.gov/nucleotide/AC023691.3?report=genbank&amp;log$=nucltop&amp;blast_rank=1&amp;RID=Y8H1SGVM016" xr:uid="{FF9FD745-ADE7-0543-B333-5A64AD1AFCD1}"/>
+    <hyperlink ref="D2" r:id="rId3" location="alnHdr_18030094" tooltip="Go to alignment for Drosophila melanogaster X BAC RP98-12H1 (Roswell Park Cancer Institute Drosophila BAC Library) complete sequence" display="https://blast.ncbi.nlm.nih.gov/Blast.cgi - alnHdr_18030094" xr:uid="{35A72727-0F31-EB49-A33C-493C05FE64C0}"/>
+    <hyperlink ref="E2" r:id="rId4" tooltip="Show report for AC023691.3" display="https://www.ncbi.nlm.nih.gov/nucleotide/AC023691.3?report=genbank&amp;log$=nucltop&amp;blast_rank=1&amp;RID=Y8H1SGVM016" xr:uid="{ACE27A35-C5F3-4244-9DD6-E2EDFB29D6EF}"/>
+    <hyperlink ref="D6" r:id="rId5" location="alnHdr_18030094" tooltip="Go to alignment for Drosophila melanogaster X BAC RP98-12H1 (Roswell Park Cancer Institute Drosophila BAC Library) complete sequence" display="https://blast.ncbi.nlm.nih.gov/Blast.cgi - alnHdr_18030094" xr:uid="{1D19C74D-514E-6D4F-8FBE-951377D18487}"/>
+    <hyperlink ref="E6" r:id="rId6" tooltip="Show report for AC023691.3" display="https://www.ncbi.nlm.nih.gov/nucleotide/AC023691.3?report=genbank&amp;log$=nucltop&amp;blast_rank=1&amp;RID=Y8H1SGVM016" xr:uid="{76E72D98-6C66-2A48-B614-C97D0382AF83}"/>
+    <hyperlink ref="D12" r:id="rId7" location="alnHdr_18030094" tooltip="Go to alignment for Drosophila melanogaster X BAC RP98-12H1 (Roswell Park Cancer Institute Drosophila BAC Library) complete sequence" display="https://blast.ncbi.nlm.nih.gov/Blast.cgi - alnHdr_18030094" xr:uid="{C1AF12BC-A441-5F4A-AF14-7DF32AD0C878}"/>
+    <hyperlink ref="E12" r:id="rId8" tooltip="Show report for AC023691.3" display="https://www.ncbi.nlm.nih.gov/nucleotide/AC023691.3?report=genbank&amp;log$=nucltop&amp;blast_rank=1&amp;RID=Y8H1SGVM016" xr:uid="{088DFF80-1E7A-C740-BBC5-1CBA8E10CB8F}"/>
+    <hyperlink ref="D13" r:id="rId9" location="alnHdr_18030094" tooltip="Go to alignment for Drosophila melanogaster X BAC RP98-12H1 (Roswell Park Cancer Institute Drosophila BAC Library) complete sequence" display="https://blast.ncbi.nlm.nih.gov/Blast.cgi - alnHdr_18030094" xr:uid="{C34D165D-C6EF-2940-80CA-8F8EBB376FE0}"/>
+    <hyperlink ref="E13" r:id="rId10" tooltip="Show report for AC023691.3" display="https://www.ncbi.nlm.nih.gov/nucleotide/AC023691.3?report=genbank&amp;log$=nucltop&amp;blast_rank=1&amp;RID=Y8H1SGVM016" xr:uid="{D7B8E92B-5AD0-DD43-BD30-60B1FFD31802}"/>
+    <hyperlink ref="D14" r:id="rId11" location="alnHdr_18030094" tooltip="Go to alignment for Drosophila melanogaster X BAC RP98-12H1 (Roswell Park Cancer Institute Drosophila BAC Library) complete sequence" display="https://blast.ncbi.nlm.nih.gov/Blast.cgi - alnHdr_18030094" xr:uid="{D7176C5C-4A1B-AB43-B970-B3BFA1CB5B5D}"/>
+    <hyperlink ref="E14" r:id="rId12" tooltip="Show report for AC023691.3" display="https://www.ncbi.nlm.nih.gov/nucleotide/AC023691.3?report=genbank&amp;log$=nucltop&amp;blast_rank=1&amp;RID=Y8H1SGVM016" xr:uid="{10AB0DFA-BA5A-4642-80E6-09785AC27A75}"/>
+    <hyperlink ref="E9" r:id="rId13" tooltip="Show report for OR729115.1" display="https://www.ncbi.nlm.nih.gov/nucleotide/OR729115.1?report=genbank&amp;log$=nucltop&amp;blast_rank=2&amp;RID=Y8H3393W016" xr:uid="{60E98894-8BBC-4044-B234-D64C611137F9}"/>
+    <hyperlink ref="D9" r:id="rId14" location="alnHdr_2600986764" tooltip="Go to alignment for MAG: Galbut virus isolate MD_FoCo21_19 segment RNA1, complete sequence" display="https://blast.ncbi.nlm.nih.gov/Blast.cgi - alnHdr_2600986764" xr:uid="{154DFE20-F10A-3C44-90A9-408812E41C4E}"/>
+    <hyperlink ref="D4" r:id="rId15" location="alnHdr_18030094" tooltip="Go to alignment for Drosophila melanogaster X BAC RP98-12H1 (Roswell Park Cancer Institute Drosophila BAC Library) complete sequence" display="https://blast.ncbi.nlm.nih.gov/Blast.cgi - alnHdr_18030094" xr:uid="{A2E8AB7F-C987-9F4B-8599-87D70F6C829C}"/>
+    <hyperlink ref="E4" r:id="rId16" tooltip="Show report for AC023691.3" display="https://www.ncbi.nlm.nih.gov/nucleotide/AC023691.3?report=genbank&amp;log$=nucltop&amp;blast_rank=1&amp;RID=Y8H1SGVM016" xr:uid="{DF876907-601F-344A-92B7-FE2DEB6E62D9}"/>
+    <hyperlink ref="D7" r:id="rId17" location="alnHdr_18030094" tooltip="Go to alignment for Drosophila melanogaster X BAC RP98-12H1 (Roswell Park Cancer Institute Drosophila BAC Library) complete sequence" display="https://blast.ncbi.nlm.nih.gov/Blast.cgi - alnHdr_18030094" xr:uid="{F2A4F3F2-C90D-DA41-BE33-F4CF1B13A0BC}"/>
+    <hyperlink ref="E7" r:id="rId18" tooltip="Show report for AC023691.3" display="https://www.ncbi.nlm.nih.gov/nucleotide/AC023691.3?report=genbank&amp;log$=nucltop&amp;blast_rank=1&amp;RID=Y8H1SGVM016" xr:uid="{42804FC7-F27B-C944-B79F-10CC2BF6CDE2}"/>
+    <hyperlink ref="D10" r:id="rId19" location="alnHdr_18030094" tooltip="Go to alignment for Drosophila melanogaster X BAC RP98-12H1 (Roswell Park Cancer Institute Drosophila BAC Library) complete sequence" display="https://blast.ncbi.nlm.nih.gov/Blast.cgi - alnHdr_18030094" xr:uid="{6288A2AD-4A21-AF49-AD62-3467CB828546}"/>
+    <hyperlink ref="E10" r:id="rId20" tooltip="Show report for AC023691.3" display="https://www.ncbi.nlm.nih.gov/nucleotide/AC023691.3?report=genbank&amp;log$=nucltop&amp;blast_rank=1&amp;RID=Y8H1SGVM016" xr:uid="{8CBBF05B-8AF8-7F4C-8F3D-FD871E3C0D23}"/>
+    <hyperlink ref="D11" r:id="rId21" location="alnHdr_18030094" tooltip="Go to alignment for Drosophila melanogaster X BAC RP98-12H1 (Roswell Park Cancer Institute Drosophila BAC Library) complete sequence" display="https://blast.ncbi.nlm.nih.gov/Blast.cgi - alnHdr_18030094" xr:uid="{6E9397E0-8DD2-D549-87FF-FAE3DA557EF8}"/>
+    <hyperlink ref="E11" r:id="rId22" tooltip="Show report for AC023691.3" display="https://www.ncbi.nlm.nih.gov/nucleotide/AC023691.3?report=genbank&amp;log$=nucltop&amp;blast_rank=1&amp;RID=Y8H1SGVM016" xr:uid="{9032DBBB-9878-904B-BF6F-918B031C8494}"/>
+    <hyperlink ref="D15" r:id="rId23" location="alnHdr_2714662214" tooltip="Go to alignment for Galbut virus isolate 1004283 putative RNA-dependent RNA polymerase gene, complete cds" display="https://blast.ncbi.nlm.nih.gov/Blast.cgi - alnHdr_2714662214" xr:uid="{2B20BA1B-A368-AD48-83C2-B6F5CBC67849}"/>
+    <hyperlink ref="E15" r:id="rId24" tooltip="Show report for OR820569.1" display="https://www.ncbi.nlm.nih.gov/nucleotide/OR820569.1?report=genbank&amp;log$=nucltop&amp;blast_rank=1&amp;RID=Y8H6FZFN016" xr:uid="{347C6090-7BB3-7D44-8F53-578FEC38E5B4}"/>
+    <hyperlink ref="D5" r:id="rId25" location="alnHdr_21539151" tooltip="Go to alignment for Drosophila melanogaster 3L BAC RP98-26L14 (Roswell Park Cancer Institute Drosophila BAC Library) complete sequence" display="https://blast.ncbi.nlm.nih.gov/Blast.cgi - alnHdr_21539151" xr:uid="{9D580FDD-FE83-494B-8452-1AF5947BE4C3}"/>
+    <hyperlink ref="E5" r:id="rId26" tooltip="Show report for AC010058.7" display="https://www.ncbi.nlm.nih.gov/nucleotide/AC010058.7?report=genbank&amp;log$=nucltop&amp;blast_rank=1&amp;RID=Y8H7SAEP016" xr:uid="{D03C2D3B-EE13-F54B-A22A-A490AB532AA1}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId27"/>
+</worksheet>
 </file>
</xml_diff>